<commit_message>
Publie la construction Salome v2
</commit_message>
<xml_diff>
--- a/géometrie vanne/parametres_vanne.xlsx
+++ b/géometrie vanne/parametres_vanne.xlsx
@@ -8,19 +8,32 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rapha\Documents\A&amp;M\stage\codex\géometrie vanne\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C60841AF-D05A-4E99-96FF-ACDA2D152FB0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6F6FC403-1316-4185-A252-E4424923BE34}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="16220" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="parametres" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="11">
   <si>
     <t>parametre</t>
   </si>
@@ -46,7 +59,13 @@
     <t>rapport_basculement</t>
   </si>
   <si>
-    <t>Circulaire</t>
+    <t>position_vanne</t>
+  </si>
+  <si>
+    <t>Ovoide</t>
+  </si>
+  <si>
+    <t>fermee</t>
   </si>
 </sst>
 </file>
@@ -907,7 +926,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B7"/>
+  <dimension ref="A1:B8"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.35">
@@ -923,7 +942,7 @@
         <v>2</v>
       </c>
       <c r="B2" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.35">
@@ -931,7 +950,7 @@
         <v>3</v>
       </c>
       <c r="B3">
-        <v>1.5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.35">
@@ -939,7 +958,7 @@
         <v>4</v>
       </c>
       <c r="B4">
-        <v>0.15</v>
+        <v>0.35</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.35">
@@ -955,7 +974,7 @@
         <v>6</v>
       </c>
       <c r="B6">
-        <v>0.6</v>
+        <v>0.7</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.35">
@@ -963,13 +982,24 @@
         <v>7</v>
       </c>
       <c r="B7">
-        <v>0.8</v>
+        <v>0.9</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A8" t="s">
+        <v>8</v>
+      </c>
+      <c r="B8" t="s">
+        <v>10</v>
       </c>
     </row>
   </sheetData>
-  <dataValidations count="1">
+  <dataValidations count="2">
     <dataValidation type="list" showErrorMessage="1" sqref="B2" xr:uid="{00000000-0002-0000-0000-000000000000}">
-      <formula1>"Ovoïde,Circulaire"</formula1>
+      <formula1>"Ovoide,Circulaire"</formula1>
+    </dataValidation>
+    <dataValidation type="list" showErrorMessage="1" sqref="B8" xr:uid="{00000000-0002-0000-0000-000001000000}">
+      <formula1>"ouverte,fermee"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>